<commit_message>
Add alternative return flight options for passengers 2 and 3
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TdiRuVNea7SeBm9dzobFft
</commit_message>
<xml_diff>
--- a/Flight_Booking_Summary_BKK-PVG.xlsx
+++ b/Flight_Booking_Summary_BKK-PVG.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -163,6 +163,7 @@
     <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -529,21 +530,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,50 +568,55 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
+          <t>Option</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>Flight No.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Departure</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Arrival</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Arrival Date</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Fare (THB/pax)</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Baggage</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Conditions</t>
         </is>
@@ -624,50 +631,51 @@
           <t>Phuriwat Jantapetch</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>MU8654</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>BKK-PVG</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>05:05</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="J4" s="7" t="n">
+      <c r="K4" s="7" t="n">
         <v>15780</v>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>1 pc (23 kg)</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
         </is>
@@ -676,44 +684,45 @@
     <row r="5">
       <c r="A5" s="8" t="n"/>
       <c r="B5" s="8" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>MU 547</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Z</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>31 AUG 2026</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>PVG-BKK</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>21:15</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>00:40</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>01 SEP 2026</t>
         </is>
       </c>
-      <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
+      <c r="M5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -724,223 +733,446 @@
           <t>Pongnut Yungyuentrakoon</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Option A</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>MU8654</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>BKK-PVG</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>05:05</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="J6" s="13" t="n">
+      <c r="K6" s="13" t="n">
         <v>17230</v>
       </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="L6" s="10" t="inlineStr">
         <is>
           <t>1 pc (23 kg)</t>
         </is>
       </c>
-      <c r="L6" s="10" t="inlineStr">
+      <c r="M6" s="10" t="inlineStr">
         <is>
           <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Refund 4,500 THB for unused ticket</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="A7" s="14" t="n"/>
+      <c r="B7" s="14" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>FM 839</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t>05 SEP 2026</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr">
         <is>
           <t>PVG-BKK</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>17:20</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="I7" s="11" t="inlineStr">
         <is>
           <t>20:55</t>
         </is>
       </c>
-      <c r="I7" s="11" t="inlineStr">
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>05 SEP 2026</t>
         </is>
       </c>
-      <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
+      <c r="M7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Kampanart Tanpithaksidh</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>FM 848</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>31 AUG 2026</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="A8" s="14" t="n"/>
+      <c r="B8" s="14" t="n"/>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Option B</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>MU8654</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>23 AUG 2026</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>BKK-PVG</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>05:05</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>10:35</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>31 AUG 2026</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>11070</v>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>23 AUG 2026</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="n">
+        <v>17230</v>
+      </c>
+      <c r="L8" s="10" t="inlineStr">
         <is>
           <t>1 pc (23 kg)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Refund 4,500 THB for unused ticket (ราคาเดียวกับ Option A)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="8" t="n"/>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>MU 547</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>05 SEP 2026</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>PVG-BKK</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>21:15</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="11" t="inlineStr">
         <is>
           <t>00:40</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="J9" s="11" t="inlineStr">
         <is>
           <t>06 SEP 2026</t>
         </is>
       </c>
-      <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
+      <c r="M9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Kampanart Tanpithaksidh</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Option A</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>FM 848</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>31 AUG 2026</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>BKK-PVG</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>05:05</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>31 AUG 2026</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>11070</v>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>1 pc (23 kg)</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Note: Fares are per passenger in THB, as quoted by the ticketing agent (user-provided). Flight change fee 2,000 THB + fare difference applies to all tickets. Arrival next day where arrival date differs from departure date.</t>
+      <c r="A11" s="14" t="n"/>
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>MU 547</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>05 SEP 2026</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>PVG-BKK</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>00:40</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>06 SEP 2026</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="8" t="n"/>
+      <c r="M11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n"/>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Option B</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>FM 848</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>31 AUG 2026</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>BKK-PVG</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>05:05</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>31 AUG 2026</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>10110</v>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>1 pc (23 kg)</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>FM 839</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>05 SEP 2026</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>PVG-BKK</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>17:20</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>05 SEP 2026</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="n"/>
+      <c r="L13" s="8" t="n"/>
+      <c r="M13" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Note: Fares are per passenger in THB, as quoted by the ticketing agent (user-provided). Pax 2: Option B (MU 547 return) is the same fare as Option A. Pax 3: Option B (FM 839 return) is THB 10,110 vs THB 11,070 for Option A. Flight change fee 2,000 THB + fare difference applies to all tickets. Arrival next day where arrival date differs from departure date.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A11:L11"/>
-    <mergeCell ref="A8:A9"/>
+  <mergeCells count="28">
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="M10:M11"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="M12:M13"/>
+    <mergeCell ref="A15:M15"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="L10:L11"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="M4:M5"/>
     <mergeCell ref="B4:B5"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="L6:L7"/>
-    <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:K7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Select latest return flight MU 547 for passengers 2 and 3
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TdiRuVNea7SeBm9dzobFft
</commit_message>
<xml_diff>
--- a/Flight_Booking_Summary_BKK-PVG.xlsx
+++ b/Flight_Booking_Summary_BKK-PVG.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -163,7 +163,6 @@
     <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -530,22 +529,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -568,55 +566,50 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Option</t>
+          <t>Flight No.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Flight No.</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Class</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Route</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Route</t>
+          <t>Departure</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Departure</t>
+          <t>Arrival</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Arrival</t>
+          <t>Arrival Date</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Arrival Date</t>
+          <t>Fare (THB/pax)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Fare (THB/pax)</t>
+          <t>Baggage</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Baggage</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Conditions</t>
         </is>
@@ -631,51 +624,50 @@
           <t>Phuriwat Jantapetch</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>MU8654</t>
+        </is>
+      </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>MU8654</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>BKK-PVG</t>
         </is>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>05:05</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>05:05</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="K4" s="7" t="n">
+      <c r="J4" s="7" t="n">
         <v>15780</v>
       </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>1 pc (23 kg)</t>
+        </is>
+      </c>
       <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>1 pc (23 kg)</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
         </is>
@@ -684,45 +676,44 @@
     <row r="5">
       <c r="A5" s="8" t="n"/>
       <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>MU 547</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>MU 547</t>
+          <t>Z</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Z</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
           <t>31 AUG 2026</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>PVG-BKK</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>00:40</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
           <t>01 SEP 2026</t>
         </is>
       </c>
+      <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="n">
@@ -733,446 +724,223 @@
           <t>Pongnut Yungyuentrakoon</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Option A</t>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>MU8654</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>MU8654</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>BKK-PVG</t>
         </is>
       </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>05:05</t>
+        </is>
+      </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>05:05</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
           <t>23 AUG 2026</t>
         </is>
       </c>
-      <c r="K6" s="13" t="n">
+      <c r="J6" s="13" t="n">
         <v>17230</v>
       </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>1 pc (23 kg)</t>
+        </is>
+      </c>
       <c r="L6" s="10" t="inlineStr">
-        <is>
-          <t>1 pc (23 kg)</t>
-        </is>
-      </c>
-      <c r="M6" s="10" t="inlineStr">
         <is>
           <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Refund 4,500 THB for unused ticket</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n"/>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="8" t="n"/>
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>MU 547</t>
+        </is>
+      </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>FM 839</t>
+          <t>T</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
           <t>05 SEP 2026</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>PVG-BKK</t>
         </is>
       </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>00:40</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>20:55</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>05 SEP 2026</t>
-        </is>
-      </c>
+          <t>06 SEP 2026</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="n"/>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Option B</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>MU8654</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>23 AUG 2026</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="A8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Kampanart Tanpithaksidh</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>FM 848</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>31 AUG 2026</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>BKK-PVG</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>05:05</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>23 AUG 2026</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>17230</v>
-      </c>
-      <c r="L8" s="10" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>31 AUG 2026</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>11070</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>1 pc (23 kg)</t>
         </is>
       </c>
-      <c r="M8" s="10" t="inlineStr">
-        <is>
-          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Refund 4,500 THB for unused ticket (ราคาเดียวกับ Option A)</t>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>MU 547</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>05 SEP 2026</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>PVG-BKK</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>21:15</t>
         </is>
       </c>
-      <c r="I9" s="11" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>00:40</t>
         </is>
       </c>
-      <c r="J9" s="11" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>06 SEP 2026</t>
         </is>
       </c>
+      <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
-      <c r="M9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Kampanart Tanpithaksidh</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Option A</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>FM 848</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>31 AUG 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>BKK-PVG</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>05:05</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>10:35</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>31 AUG 2026</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>11070</v>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>1 pc (23 kg)</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
-        </is>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>MU 547</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>05 SEP 2026</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>PVG-BKK</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>21:15</t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>00:40</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>06 SEP 2026</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="8" t="n"/>
-      <c r="M11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Option B</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>FM 848</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>31 AUG 2026</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>BKK-PVG</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>05:05</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>10:35</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>31 AUG 2026</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>10110</v>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>1 pc (23 kg)</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>เปลี่ยนไฟล์ท 2,000฿ + ส่วนต่าง / Non-refundable</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>FM 839</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>T</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>05 SEP 2026</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>PVG-BKK</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>17:20</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>20:55</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>05 SEP 2026</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="8" t="n"/>
-      <c r="M13" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Note: Fares are per passenger in THB, as quoted by the ticketing agent (user-provided). Pax 2: Option B (MU 547 return) is the same fare as Option A. Pax 3: Option B (FM 839 return) is THB 10,110 vs THB 11,070 for Option A. Flight change fee 2,000 THB + fare difference applies to all tickets. Arrival next day where arrival date differs from departure date.</t>
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Note: Fares are per passenger in THB, as quoted by the ticketing agent (user-provided). Pax 2 and 3 selected the latest return flight (MU 547, dep 21:15) per traveler preference; MU 547 arrives BKK next day at 00:40. Flight change fee 2,000 THB + fare difference applies to all tickets.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="L12:L13"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="M10:M11"/>
+  <mergeCells count="17">
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="L8:L9"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="K4:K5"/>
     <mergeCell ref="L4:L5"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="M12:M13"/>
-    <mergeCell ref="A15:M15"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="L10:L11"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="B6:B9"/>
     <mergeCell ref="L6:L7"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:K7"/>
-    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>